<commit_message>
Add security guards comparison PDF; fix OMC guard counts in workbook
Exclude station security supervisors from OMC guard totals and include
P&R guards at their host station so both reports use the same method.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VswDpGdrhaaM8XdvXVqV99
</commit_message>
<xml_diff>
--- a/Riyadh_Metro_vs_OMC_Differences.xlsx
+++ b/Riyadh_Metro_vs_OMC_Differences.xlsx
@@ -160,7 +160,7 @@
     <t xml:space="preserve">SecG Total/day</t>
   </si>
   <si>
-    <t xml:space="preserve">OMC SecG per shift</t>
+    <t xml:space="preserve">OMC SecG per shift (incl. P&amp;R)</t>
   </si>
   <si>
     <t xml:space="preserve">Diff (OMC − E-shift)</t>
@@ -1841,31 +1841,31 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">SUMPRODUCT((Comparison!$B$3:$B$94="Line 1")*ISNUMBER(Comparison!$AC$3:$AC$94)*(Comparison!$AC$3:$AC$94&lt;&gt;0))</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">SUMPRODUCT((Comparison!$B$3:$B$94="Line 2")*ISNUMBER(Comparison!$AC$3:$AC$94)*(Comparison!$AC$3:$AC$94&lt;&gt;0))</f>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">SUMPRODUCT((Comparison!$B$3:$B$94="Line 3")*ISNUMBER(Comparison!$AC$3:$AC$94)*(Comparison!$AC$3:$AC$94&lt;&gt;0))</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">SUMPRODUCT((Comparison!$B$3:$B$94="Line 4")*ISNUMBER(Comparison!$AC$3:$AC$94)*(Comparison!$AC$3:$AC$94&lt;&gt;0))</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F10" s="5" t="n">
         <f aca="false">SUMPRODUCT((Comparison!$B$3:$B$94="Line 5")*ISNUMBER(Comparison!$AC$3:$AC$94)*(Comparison!$AC$3:$AC$94&lt;&gt;0))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10" s="5" t="n">
         <f aca="false">SUMPRODUCT((Comparison!$B$3:$B$94="Line 6")*ISNUMBER(Comparison!$AC$3:$AC$94)*(Comparison!$AC$3:$AC$94&lt;&gt;0))</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H10" s="5" t="n">
         <f aca="false">SUM(B10:G10)</f>
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2192,11 +2192,11 @@
         <v>5</v>
       </c>
       <c r="AB3" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC3" s="12" t="n">
         <f aca="false">IF(AND(X3="",AB3=0),"",N(AB3)-N(X3))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD3" s="10" t="n">
         <f aca="false">COUNTIF(H3:W3,"✗")</f>
@@ -4348,11 +4348,11 @@
         <v>7</v>
       </c>
       <c r="AB25" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AC25" s="12" t="n">
         <f aca="false">IF(AND(X25="",AB25=0),"",N(AB25)-N(X25))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD25" s="10" t="n">
         <f aca="false">COUNTIF(H25:W25,"✗")</f>
@@ -4548,11 +4548,11 @@
         <v>7</v>
       </c>
       <c r="AB27" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AC27" s="12" t="n">
         <f aca="false">IF(AND(X27="",AB27=0),"",N(AB27)-N(X27))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD27" s="10" t="n">
         <f aca="false">COUNTIF(H27:W27,"✗")</f>
@@ -6048,11 +6048,11 @@
         <v>7</v>
       </c>
       <c r="AB42" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC42" s="12" t="n">
         <f aca="false">IF(AND(X42="",AB42=0),"",N(AB42)-N(X42))</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AD42" s="10" t="n">
         <f aca="false">COUNTIF(H42:W42,"✗")</f>
@@ -6148,11 +6148,11 @@
         <v>7</v>
       </c>
       <c r="AB43" s="10" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="AC43" s="12" t="n">
         <f aca="false">IF(AND(X43="",AB43=0),"",N(AB43)-N(X43))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AD43" s="10" t="n">
         <f aca="false">COUNTIF(H43:W43,"✗")</f>
@@ -6442,11 +6442,11 @@
         <v>10</v>
       </c>
       <c r="AB46" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AC46" s="12" t="n">
         <f aca="false">IF(AND(X46="",AB46=0),"",N(AB46)-N(X46))</f>
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AD46" s="10" t="n">
         <f aca="false">COUNTIF(H46:W46,"✗")</f>
@@ -6742,11 +6742,11 @@
         <v>7</v>
       </c>
       <c r="AB49" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC49" s="12" t="n">
         <f aca="false">IF(AND(X49="",AB49=0),"",N(AB49)-N(X49))</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AD49" s="10" t="n">
         <f aca="false">COUNTIF(H49:W49,"✗")</f>
@@ -7042,11 +7042,11 @@
         <v>8</v>
       </c>
       <c r="AB52" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AC52" s="12" t="n">
         <f aca="false">IF(AND(X52="",AB52=0),"",N(AB52)-N(X52))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD52" s="10" t="n">
         <f aca="false">COUNTIF(H52:W52,"✗")</f>
@@ -7642,11 +7642,11 @@
         <v>3</v>
       </c>
       <c r="AB58" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC58" s="12" t="n">
         <f aca="false">IF(AND(X58="",AB58=0),"",N(AB58)-N(X58))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD58" s="10" t="n">
         <f aca="false">COUNTIF(H58:W58,"✗")</f>
@@ -7842,11 +7842,11 @@
         <v>9</v>
       </c>
       <c r="AB60" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC60" s="12" t="n">
         <f aca="false">IF(AND(X60="",AB60=0),"",N(AB60)-N(X60))</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AD60" s="10" t="n">
         <f aca="false">COUNTIF(H60:W60,"✗")</f>
@@ -8236,11 +8236,11 @@
         <v>7</v>
       </c>
       <c r="AB64" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC64" s="12" t="n">
         <f aca="false">IF(AND(X64="",AB64=0),"",N(AB64)-N(X64))</f>
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AD64" s="10" t="n">
         <f aca="false">COUNTIF(H64:W64,"✗")</f>
@@ -8416,11 +8416,11 @@
         <v>6</v>
       </c>
       <c r="AB66" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AC66" s="12" t="n">
         <f aca="false">IF(AND(X66="",AB66=0),"",N(AB66)-N(X66))</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AD66" s="10" t="n">
         <f aca="false">COUNTIF(H66:W66,"✗")</f>
@@ -8816,11 +8816,11 @@
         <v>9</v>
       </c>
       <c r="AB70" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC70" s="12" t="n">
         <f aca="false">IF(AND(X70="",AB70=0),"",N(AB70)-N(X70))</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AD70" s="10" t="n">
         <f aca="false">COUNTIF(H70:W70,"✗")</f>
@@ -10216,11 +10216,11 @@
         <v>3</v>
       </c>
       <c r="AB84" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC84" s="12" t="n">
         <f aca="false">IF(AND(X84="",AB84=0),"",N(AB84)-N(X84))</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AD84" s="10" t="n">
         <f aca="false">COUNTIF(H84:W84,"✗")</f>
@@ -10550,11 +10550,11 @@
         <v>4</v>
       </c>
       <c r="AB88" s="10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AC88" s="12" t="n">
         <f aca="false">IF(AND(X88="",AB88=0),"",N(AB88)-N(X88))</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AD88" s="10" t="n">
         <f aca="false">COUNTIF(H88:W88,"✗")</f>
@@ -10750,11 +10750,11 @@
         <v>13</v>
       </c>
       <c r="AB90" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AC90" s="12" t="n">
         <f aca="false">IF(AND(X90="",AB90=0),"",N(AB90)-N(X90))</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AD90" s="10" t="n">
         <f aca="false">COUNTIF(H90:W90,"✗")</f>
@@ -11136,11 +11136,11 @@
         <v>5</v>
       </c>
       <c r="AB94" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC94" s="12" t="n">
         <f aca="false">IF(AND(X94="",AB94=0),"",N(AB94)-N(X94))</f>
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AD94" s="10" t="n">
         <f aca="false">COUNTIF(H94:W94,"✗")</f>

</xml_diff>